<commit_message>
save before moving onto the agentic
</commit_message>
<xml_diff>
--- a/task_graph/referring_expression_responses.xlsx
+++ b/task_graph/referring_expression_responses.xlsx
@@ -177,7 +177,7 @@
       </c>
       <c r="F5" t="inlineStr" s="0">
         <is>
-          <t>BaseBoard</t>
+          <t>BASE_BOARD</t>
         </is>
       </c>
       <c r="G5" t="inlineStr" s="0">
@@ -244,7 +244,7 @@
       </c>
       <c r="F6" t="inlineStr" s="0">
         <is>
-          <t>BaseBoard</t>
+          <t>BASE_BOARD</t>
         </is>
       </c>
       <c r="G6" t="inlineStr" s="0">
@@ -311,7 +311,7 @@
       </c>
       <c r="F7" t="inlineStr" s="0">
         <is>
-          <t>BaseBoard</t>
+          <t>BASE_BOARD</t>
         </is>
       </c>
       <c r="G7" t="inlineStr" s="0">
@@ -378,7 +378,7 @@
       </c>
       <c r="F8" t="inlineStr" s="0">
         <is>
-          <t>BaseBoard</t>
+          <t>BASE_BOARD</t>
         </is>
       </c>
       <c r="G8" t="inlineStr" s="0">
@@ -445,7 +445,7 @@
       </c>
       <c r="F9" t="inlineStr" s="0">
         <is>
-          <t>BaseBoard</t>
+          <t>BASE_BOARD</t>
         </is>
       </c>
       <c r="G9" t="inlineStr" s="0">
@@ -512,7 +512,7 @@
       </c>
       <c r="F10" t="inlineStr" s="0">
         <is>
-          <t>BaseBoard</t>
+          <t>BASE_BOARD</t>
         </is>
       </c>
       <c r="G10" t="inlineStr" s="0">
@@ -579,7 +579,7 @@
       </c>
       <c r="F11" t="inlineStr" s="0">
         <is>
-          <t>BaseBoard</t>
+          <t>BASE_BOARD</t>
         </is>
       </c>
       <c r="G11" t="inlineStr" s="0">
@@ -646,7 +646,7 @@
       </c>
       <c r="F12" t="inlineStr" s="0">
         <is>
-          <t>BaseBoard</t>
+          <t>BASE_BOARD</t>
         </is>
       </c>
       <c r="G12" t="inlineStr" s="0">
@@ -713,7 +713,7 @@
       </c>
       <c r="F13" t="inlineStr" s="0">
         <is>
-          <t>BaseBoard</t>
+          <t>BASE_BOARD</t>
         </is>
       </c>
       <c r="G13" t="inlineStr" s="0">
@@ -780,7 +780,7 @@
       </c>
       <c r="F14" t="inlineStr" s="0">
         <is>
-          <t>BaseBoard</t>
+          <t>BASE_BOARD</t>
         </is>
       </c>
       <c r="G14" t="inlineStr" s="0">
@@ -847,7 +847,7 @@
       </c>
       <c r="F15" t="inlineStr" s="0">
         <is>
-          <t>Bearing</t>
+          <t>BEARING</t>
         </is>
       </c>
       <c r="G15" t="inlineStr" s="0">
@@ -914,7 +914,7 @@
       </c>
       <c r="F16" t="inlineStr" s="0">
         <is>
-          <t>Bearing</t>
+          <t>BEARING</t>
         </is>
       </c>
       <c r="G16" t="inlineStr" s="0">
@@ -981,7 +981,7 @@
       </c>
       <c r="F17" t="inlineStr" s="0">
         <is>
-          <t>Bearing</t>
+          <t>BEARING</t>
         </is>
       </c>
       <c r="G17" t="inlineStr" s="0">
@@ -1048,7 +1048,7 @@
       </c>
       <c r="F18" t="inlineStr" s="0">
         <is>
-          <t>Bearing</t>
+          <t>BEARING</t>
         </is>
       </c>
       <c r="G18" t="inlineStr" s="0">
@@ -1115,7 +1115,7 @@
       </c>
       <c r="F19" t="inlineStr" s="0">
         <is>
-          <t>Bearing</t>
+          <t>BEARING</t>
         </is>
       </c>
       <c r="G19" t="inlineStr" s="0">
@@ -1182,7 +1182,7 @@
       </c>
       <c r="F20" t="inlineStr" s="0">
         <is>
-          <t>Bearing</t>
+          <t>BEARING</t>
         </is>
       </c>
       <c r="G20" t="inlineStr" s="0">
@@ -1249,7 +1249,7 @@
       </c>
       <c r="F21" t="inlineStr" s="0">
         <is>
-          <t>Bearing</t>
+          <t>BEARING</t>
         </is>
       </c>
       <c r="G21" t="inlineStr" s="0">
@@ -1316,7 +1316,7 @@
       </c>
       <c r="F22" t="inlineStr" s="0">
         <is>
-          <t>Bearing</t>
+          <t>BEARING</t>
         </is>
       </c>
       <c r="G22" t="inlineStr" s="0">
@@ -1383,7 +1383,7 @@
       </c>
       <c r="F23" t="inlineStr" s="0">
         <is>
-          <t>Bearing</t>
+          <t>BEARING</t>
         </is>
       </c>
       <c r="G23" t="inlineStr" s="0">
@@ -1450,7 +1450,7 @@
       </c>
       <c r="F24" t="inlineStr" s="0">
         <is>
-          <t>Bearing</t>
+          <t>BEARING</t>
         </is>
       </c>
       <c r="G24" t="inlineStr" s="0">
@@ -1517,7 +1517,7 @@
       </c>
       <c r="F25" t="inlineStr" s="0">
         <is>
-          <t>Handle</t>
+          <t>CRANK_HANDLE_ROW1</t>
         </is>
       </c>
       <c r="G25" t="inlineStr" s="0">
@@ -1584,7 +1584,7 @@
       </c>
       <c r="F26" t="inlineStr" s="0">
         <is>
-          <t>Handle</t>
+          <t>CRANK_HANDLE_ROW1</t>
         </is>
       </c>
       <c r="G26" t="inlineStr" s="0">
@@ -1651,7 +1651,7 @@
       </c>
       <c r="F27" t="inlineStr" s="0">
         <is>
-          <t>Handle</t>
+          <t>CRANK_HANDLE_ROW1</t>
         </is>
       </c>
       <c r="G27" t="inlineStr" s="0">
@@ -1718,7 +1718,7 @@
       </c>
       <c r="F28" t="inlineStr" s="0">
         <is>
-          <t>Handle</t>
+          <t>CRANK_HANDLE_ROW1</t>
         </is>
       </c>
       <c r="G28" t="inlineStr" s="0">
@@ -1785,7 +1785,7 @@
       </c>
       <c r="F29" t="inlineStr" s="0">
         <is>
-          <t>Handle</t>
+          <t>CRANK_HANDLE_ROW1</t>
         </is>
       </c>
       <c r="G29" t="inlineStr" s="0">
@@ -1852,7 +1852,7 @@
       </c>
       <c r="F30" t="inlineStr" s="0">
         <is>
-          <t>Handle</t>
+          <t>CRANK_HANDLE_ROW1</t>
         </is>
       </c>
       <c r="G30" t="inlineStr" s="0">
@@ -1919,7 +1919,7 @@
       </c>
       <c r="F31" t="inlineStr" s="0">
         <is>
-          <t>Handle</t>
+          <t>CRANK_HANDLE_ROW1</t>
         </is>
       </c>
       <c r="G31" t="inlineStr" s="0">
@@ -1986,7 +1986,7 @@
       </c>
       <c r="F32" t="inlineStr" s="0">
         <is>
-          <t>Handle</t>
+          <t>CRANK_HANDLE_ROW1</t>
         </is>
       </c>
       <c r="G32" t="inlineStr" s="0">
@@ -2053,7 +2053,7 @@
       </c>
       <c r="F33" t="inlineStr" s="0">
         <is>
-          <t>Handle</t>
+          <t>CRANK_HANDLE_ROW1</t>
         </is>
       </c>
       <c r="G33" t="inlineStr" s="0">
@@ -2120,7 +2120,7 @@
       </c>
       <c r="F34" t="inlineStr" s="0">
         <is>
-          <t>Handle</t>
+          <t>CRANK_HANDLE_ROW1</t>
         </is>
       </c>
       <c r="G34" t="inlineStr" s="0">
@@ -2187,7 +2187,7 @@
       </c>
       <c r="F35" t="inlineStr" s="0">
         <is>
-          <t>Row1_GearRod</t>
+          <t>GEAR_ROD_ROW1</t>
         </is>
       </c>
       <c r="G35" t="inlineStr" s="0">
@@ -2254,7 +2254,7 @@
       </c>
       <c r="F36" t="inlineStr" s="0">
         <is>
-          <t>Row1_GearRod</t>
+          <t>GEAR_ROD_ROW1</t>
         </is>
       </c>
       <c r="G36" t="inlineStr" s="0">
@@ -2321,7 +2321,7 @@
       </c>
       <c r="F37" t="inlineStr" s="0">
         <is>
-          <t>Row1_GearRod</t>
+          <t>GEAR_ROD_ROW1</t>
         </is>
       </c>
       <c r="G37" t="inlineStr" s="0">
@@ -2388,7 +2388,7 @@
       </c>
       <c r="F38" t="inlineStr" s="0">
         <is>
-          <t>Row1_GearRod</t>
+          <t>GEAR_ROD_ROW1</t>
         </is>
       </c>
       <c r="G38" t="inlineStr" s="0">
@@ -2455,7 +2455,7 @@
       </c>
       <c r="F39" t="inlineStr" s="0">
         <is>
-          <t>Row1_GearRod</t>
+          <t>GEAR_ROD_ROW1</t>
         </is>
       </c>
       <c r="G39" t="inlineStr" s="0">
@@ -2522,7 +2522,7 @@
       </c>
       <c r="F40" t="inlineStr" s="0">
         <is>
-          <t>Row1_GearRod</t>
+          <t>GEAR_ROD_ROW1</t>
         </is>
       </c>
       <c r="G40" t="inlineStr" s="0">
@@ -2589,7 +2589,7 @@
       </c>
       <c r="F41" t="inlineStr" s="0">
         <is>
-          <t>Row1_GearRod</t>
+          <t>GEAR_ROD_ROW1</t>
         </is>
       </c>
       <c r="G41" t="inlineStr" s="0">
@@ -2656,7 +2656,7 @@
       </c>
       <c r="F42" t="inlineStr" s="0">
         <is>
-          <t>Row1_GearRod</t>
+          <t>GEAR_ROD_ROW1</t>
         </is>
       </c>
       <c r="G42" t="inlineStr" s="0">
@@ -2723,7 +2723,7 @@
       </c>
       <c r="F43" t="inlineStr" s="0">
         <is>
-          <t>Row1_GearRod</t>
+          <t>GEAR_ROD_ROW1</t>
         </is>
       </c>
       <c r="G43" t="inlineStr" s="0">
@@ -2790,7 +2790,7 @@
       </c>
       <c r="F44" t="inlineStr" s="0">
         <is>
-          <t>Row1_GearRod</t>
+          <t>GEAR_ROD_ROW1</t>
         </is>
       </c>
       <c r="G44" t="inlineStr" s="0">
@@ -2857,7 +2857,7 @@
       </c>
       <c r="F45" t="inlineStr" s="0">
         <is>
-          <t>Row1_GearRod</t>
+          <t>GEAR_ROD_ROW1</t>
         </is>
       </c>
       <c r="G45" t="inlineStr" s="0">
@@ -2924,7 +2924,7 @@
       </c>
       <c r="F46" t="inlineStr" s="0">
         <is>
-          <t>Row1_GearRod</t>
+          <t>GEAR_ROD_ROW1</t>
         </is>
       </c>
       <c r="G46" t="inlineStr" s="0">
@@ -2991,7 +2991,7 @@
       </c>
       <c r="F47" t="inlineStr" s="0">
         <is>
-          <t>Row1_GearStand_Left</t>
+          <t>STAND_ROW1_LEFT</t>
         </is>
       </c>
       <c r="G47" t="inlineStr" s="0">
@@ -3058,7 +3058,7 @@
       </c>
       <c r="F48" t="inlineStr" s="0">
         <is>
-          <t>Row1_GearStand_Left</t>
+          <t>STAND_ROW1_LEFT</t>
         </is>
       </c>
       <c r="G48" t="inlineStr" s="0">
@@ -3125,7 +3125,7 @@
       </c>
       <c r="F49" t="inlineStr" s="0">
         <is>
-          <t>Row1_GearStand_Left</t>
+          <t>STAND_ROW1_LEFT</t>
         </is>
       </c>
       <c r="G49" t="inlineStr" s="0">
@@ -3192,7 +3192,7 @@
       </c>
       <c r="F50" t="inlineStr" s="0">
         <is>
-          <t>Row1_GearStand_Left</t>
+          <t>STAND_ROW1_LEFT</t>
         </is>
       </c>
       <c r="G50" t="inlineStr" s="0">
@@ -3259,7 +3259,7 @@
       </c>
       <c r="F51" t="inlineStr" s="0">
         <is>
-          <t>Row1_GearStand_Left</t>
+          <t>STAND_ROW1_LEFT</t>
         </is>
       </c>
       <c r="G51" t="inlineStr" s="0">
@@ -3326,7 +3326,7 @@
       </c>
       <c r="F52" t="inlineStr" s="0">
         <is>
-          <t>Row1_GearStand_Left</t>
+          <t>STAND_ROW1_LEFT</t>
         </is>
       </c>
       <c r="G52" t="inlineStr" s="0">
@@ -3393,7 +3393,7 @@
       </c>
       <c r="F53" t="inlineStr" s="0">
         <is>
-          <t>Row1_GearStand_Left</t>
+          <t>STAND_ROW1_LEFT</t>
         </is>
       </c>
       <c r="G53" t="inlineStr" s="0">
@@ -3460,7 +3460,7 @@
       </c>
       <c r="F54" t="inlineStr" s="0">
         <is>
-          <t>Row1_GearStand_Left</t>
+          <t>STAND_ROW1_LEFT</t>
         </is>
       </c>
       <c r="G54" t="inlineStr" s="0">
@@ -3527,7 +3527,7 @@
       </c>
       <c r="F55" t="inlineStr" s="0">
         <is>
-          <t>Row1_GearStand_Left</t>
+          <t>STAND_ROW1_LEFT</t>
         </is>
       </c>
       <c r="G55" t="inlineStr" s="0">
@@ -3594,7 +3594,7 @@
       </c>
       <c r="F56" t="inlineStr" s="0">
         <is>
-          <t>Row1_GearStand_Left</t>
+          <t>STAND_ROW1_LEFT</t>
         </is>
       </c>
       <c r="G56" t="inlineStr" s="0">
@@ -3661,7 +3661,7 @@
       </c>
       <c r="F57" t="inlineStr" s="0">
         <is>
-          <t>Row1_GearStand_Left</t>
+          <t>STAND_ROW1_LEFT</t>
         </is>
       </c>
       <c r="G57" t="inlineStr" s="0">
@@ -3728,7 +3728,7 @@
       </c>
       <c r="F58" t="inlineStr" s="0">
         <is>
-          <t>Row1_GearStand_Left</t>
+          <t>STAND_ROW1_LEFT</t>
         </is>
       </c>
       <c r="G58" t="inlineStr" s="0">
@@ -3795,7 +3795,7 @@
       </c>
       <c r="F59" t="inlineStr" s="0">
         <is>
-          <t>Row1_GearStand_Right</t>
+          <t>STAND_ROW1_RIGHT</t>
         </is>
       </c>
       <c r="G59" t="inlineStr" s="0">
@@ -3862,7 +3862,7 @@
       </c>
       <c r="F60" t="inlineStr" s="0">
         <is>
-          <t>Row1_GearStand_Right</t>
+          <t>STAND_ROW1_RIGHT</t>
         </is>
       </c>
       <c r="G60" t="inlineStr" s="0">
@@ -3929,7 +3929,7 @@
       </c>
       <c r="F61" t="inlineStr" s="0">
         <is>
-          <t>Row1_GearStand_Right</t>
+          <t>STAND_ROW1_RIGHT</t>
         </is>
       </c>
       <c r="G61" t="inlineStr" s="0">
@@ -3996,7 +3996,7 @@
       </c>
       <c r="F62" t="inlineStr" s="0">
         <is>
-          <t>Row1_GearStand_Right</t>
+          <t>STAND_ROW1_RIGHT</t>
         </is>
       </c>
       <c r="G62" t="inlineStr" s="0">
@@ -4063,7 +4063,7 @@
       </c>
       <c r="F63" t="inlineStr" s="0">
         <is>
-          <t>Row1_GearStand_Right</t>
+          <t>STAND_ROW1_RIGHT</t>
         </is>
       </c>
       <c r="G63" t="inlineStr" s="0">
@@ -4130,7 +4130,7 @@
       </c>
       <c r="F64" t="inlineStr" s="0">
         <is>
-          <t>Row1_GearStand_Right</t>
+          <t>STAND_ROW1_RIGHT</t>
         </is>
       </c>
       <c r="G64" t="inlineStr" s="0">
@@ -4197,7 +4197,7 @@
       </c>
       <c r="F65" t="inlineStr" s="0">
         <is>
-          <t>Row1_GearStand_Right</t>
+          <t>STAND_ROW1_RIGHT</t>
         </is>
       </c>
       <c r="G65" t="inlineStr" s="0">
@@ -4264,7 +4264,7 @@
       </c>
       <c r="F66" t="inlineStr" s="0">
         <is>
-          <t>Row1_GearStand_Right</t>
+          <t>STAND_ROW1_RIGHT</t>
         </is>
       </c>
       <c r="G66" t="inlineStr" s="0">
@@ -4331,7 +4331,7 @@
       </c>
       <c r="F67" t="inlineStr" s="0">
         <is>
-          <t>Row1_GearStand_Right</t>
+          <t>STAND_ROW1_RIGHT</t>
         </is>
       </c>
       <c r="G67" t="inlineStr" s="0">
@@ -4398,7 +4398,7 @@
       </c>
       <c r="F68" t="inlineStr" s="0">
         <is>
-          <t>Row1_GearStand_Right</t>
+          <t>STAND_ROW1_RIGHT</t>
         </is>
       </c>
       <c r="G68" t="inlineStr" s="0">
@@ -4465,7 +4465,7 @@
       </c>
       <c r="F69" t="inlineStr" s="0">
         <is>
-          <t>Row1_GearStand_Right</t>
+          <t>STAND_ROW1_RIGHT</t>
         </is>
       </c>
       <c r="G69" t="inlineStr" s="0">
@@ -4532,7 +4532,7 @@
       </c>
       <c r="F70" t="inlineStr" s="0">
         <is>
-          <t>Row1_GearStand_Right</t>
+          <t>STAND_ROW1_RIGHT</t>
         </is>
       </c>
       <c r="G70" t="inlineStr" s="0">
@@ -4599,7 +4599,7 @@
       </c>
       <c r="F71" t="inlineStr" s="0">
         <is>
-          <t>Row1_Gear_Left</t>
+          <t>GEAR_ROW1_LEFT</t>
         </is>
       </c>
       <c r="G71" t="inlineStr" s="0">
@@ -4666,7 +4666,7 @@
       </c>
       <c r="F72" t="inlineStr" s="0">
         <is>
-          <t>Row1_Gear_Left</t>
+          <t>GEAR_ROW1_LEFT</t>
         </is>
       </c>
       <c r="G72" t="inlineStr" s="0">
@@ -4733,7 +4733,7 @@
       </c>
       <c r="F73" t="inlineStr" s="0">
         <is>
-          <t>Row1_Gear_Left</t>
+          <t>GEAR_ROW1_LEFT</t>
         </is>
       </c>
       <c r="G73" t="inlineStr" s="0">
@@ -4800,7 +4800,7 @@
       </c>
       <c r="F74" t="inlineStr" s="0">
         <is>
-          <t>Row1_Gear_Left</t>
+          <t>GEAR_ROW1_LEFT</t>
         </is>
       </c>
       <c r="G74" t="inlineStr" s="0">
@@ -4867,7 +4867,7 @@
       </c>
       <c r="F75" t="inlineStr" s="0">
         <is>
-          <t>Row1_Gear_Left</t>
+          <t>GEAR_ROW1_LEFT</t>
         </is>
       </c>
       <c r="G75" t="inlineStr" s="0">
@@ -4934,7 +4934,7 @@
       </c>
       <c r="F76" t="inlineStr" s="0">
         <is>
-          <t>Row1_Gear_Left</t>
+          <t>GEAR_ROW1_LEFT</t>
         </is>
       </c>
       <c r="G76" t="inlineStr" s="0">
@@ -5001,7 +5001,7 @@
       </c>
       <c r="F77" t="inlineStr" s="0">
         <is>
-          <t>Row1_Gear_Left</t>
+          <t>GEAR_ROW1_LEFT</t>
         </is>
       </c>
       <c r="G77" t="inlineStr" s="0">
@@ -5068,7 +5068,7 @@
       </c>
       <c r="F78" t="inlineStr" s="0">
         <is>
-          <t>Row1_Gear_Left</t>
+          <t>GEAR_ROW1_LEFT</t>
         </is>
       </c>
       <c r="G78" t="inlineStr" s="0">
@@ -5135,7 +5135,7 @@
       </c>
       <c r="F79" t="inlineStr" s="0">
         <is>
-          <t>Row1_Gear_Left</t>
+          <t>GEAR_ROW1_LEFT</t>
         </is>
       </c>
       <c r="G79" t="inlineStr" s="0">
@@ -5202,7 +5202,7 @@
       </c>
       <c r="F80" t="inlineStr" s="0">
         <is>
-          <t>Row1_Gear_Left</t>
+          <t>GEAR_ROW1_LEFT</t>
         </is>
       </c>
       <c r="G80" t="inlineStr" s="0">
@@ -5269,7 +5269,7 @@
       </c>
       <c r="F81" t="inlineStr" s="0">
         <is>
-          <t>Row1_Gear_Left</t>
+          <t>GEAR_ROW1_LEFT</t>
         </is>
       </c>
       <c r="G81" t="inlineStr" s="0">
@@ -5336,7 +5336,7 @@
       </c>
       <c r="F82" t="inlineStr" s="0">
         <is>
-          <t>Row1_Gear_Left</t>
+          <t>GEAR_ROW1_LEFT</t>
         </is>
       </c>
       <c r="G82" t="inlineStr" s="0">
@@ -5403,7 +5403,7 @@
       </c>
       <c r="F83" t="inlineStr" s="0">
         <is>
-          <t>Row1_Screws</t>
+          <t>SCREW_ROW1</t>
         </is>
       </c>
       <c r="G83" t="inlineStr" s="0">
@@ -5470,7 +5470,7 @@
       </c>
       <c r="F84" t="inlineStr" s="0">
         <is>
-          <t>Row1_Screws</t>
+          <t>SCREW_ROW1</t>
         </is>
       </c>
       <c r="G84" t="inlineStr" s="0">
@@ -5537,7 +5537,7 @@
       </c>
       <c r="F85" t="inlineStr" s="0">
         <is>
-          <t>Row1_Screws</t>
+          <t>SCREW_ROW1</t>
         </is>
       </c>
       <c r="G85" t="inlineStr" s="0">
@@ -5604,7 +5604,7 @@
       </c>
       <c r="F86" t="inlineStr" s="0">
         <is>
-          <t>Row1_Screws</t>
+          <t>SCREW_ROW1</t>
         </is>
       </c>
       <c r="G86" t="inlineStr" s="0">
@@ -5671,7 +5671,7 @@
       </c>
       <c r="F87" t="inlineStr" s="0">
         <is>
-          <t>Row1_Screws</t>
+          <t>SCREW_ROW1</t>
         </is>
       </c>
       <c r="G87" t="inlineStr" s="0">
@@ -5738,7 +5738,7 @@
       </c>
       <c r="F88" t="inlineStr" s="0">
         <is>
-          <t>Row1_Screws</t>
+          <t>SCREW_ROW1</t>
         </is>
       </c>
       <c r="G88" t="inlineStr" s="0">
@@ -5805,7 +5805,7 @@
       </c>
       <c r="F89" t="inlineStr" s="0">
         <is>
-          <t>Row1_Screws</t>
+          <t>SCREW_ROW1</t>
         </is>
       </c>
       <c r="G89" t="inlineStr" s="0">
@@ -5872,7 +5872,7 @@
       </c>
       <c r="F90" t="inlineStr" s="0">
         <is>
-          <t>Row1_Screws</t>
+          <t>SCREW_ROW1</t>
         </is>
       </c>
       <c r="G90" t="inlineStr" s="0">
@@ -5939,7 +5939,7 @@
       </c>
       <c r="F91" t="inlineStr" s="0">
         <is>
-          <t>Row1_Screws</t>
+          <t>SCREW_ROW1</t>
         </is>
       </c>
       <c r="G91" t="inlineStr" s="0">
@@ -6006,7 +6006,7 @@
       </c>
       <c r="F92" t="inlineStr" s="0">
         <is>
-          <t>Row2_GearRod</t>
+          <t>GEAR_ROD_ROW2</t>
         </is>
       </c>
       <c r="G92" t="inlineStr" s="0">
@@ -6073,7 +6073,7 @@
       </c>
       <c r="F93" t="inlineStr" s="0">
         <is>
-          <t>Row2_GearRod</t>
+          <t>GEAR_ROD_ROW2</t>
         </is>
       </c>
       <c r="G93" t="inlineStr" s="0">
@@ -6140,7 +6140,7 @@
       </c>
       <c r="F94" t="inlineStr" s="0">
         <is>
-          <t>Row2_GearRod</t>
+          <t>GEAR_ROD_ROW2</t>
         </is>
       </c>
       <c r="G94" t="inlineStr" s="0">
@@ -6207,7 +6207,7 @@
       </c>
       <c r="F95" t="inlineStr" s="0">
         <is>
-          <t>Row2_GearRod</t>
+          <t>GEAR_ROD_ROW2</t>
         </is>
       </c>
       <c r="G95" t="inlineStr" s="0">
@@ -6274,7 +6274,7 @@
       </c>
       <c r="F96" t="inlineStr" s="0">
         <is>
-          <t>Row2_GearRod</t>
+          <t>GEAR_ROD_ROW2</t>
         </is>
       </c>
       <c r="G96" t="inlineStr" s="0">
@@ -6341,7 +6341,7 @@
       </c>
       <c r="F97" t="inlineStr" s="0">
         <is>
-          <t>Row2_GearRod</t>
+          <t>GEAR_ROD_ROW2</t>
         </is>
       </c>
       <c r="G97" t="inlineStr" s="0">
@@ -6408,7 +6408,7 @@
       </c>
       <c r="F98" t="inlineStr" s="0">
         <is>
-          <t>Row2_GearRod</t>
+          <t>GEAR_ROD_ROW2</t>
         </is>
       </c>
       <c r="G98" t="inlineStr" s="0">
@@ -6475,7 +6475,7 @@
       </c>
       <c r="F99" t="inlineStr" s="0">
         <is>
-          <t>Row2_GearRod</t>
+          <t>GEAR_ROD_ROW2</t>
         </is>
       </c>
       <c r="G99" t="inlineStr" s="0">
@@ -6542,7 +6542,7 @@
       </c>
       <c r="F100" t="inlineStr" s="0">
         <is>
-          <t>Row2_GearRod</t>
+          <t>GEAR_ROD_ROW2</t>
         </is>
       </c>
       <c r="G100" t="inlineStr" s="0">
@@ -6609,7 +6609,7 @@
       </c>
       <c r="F101" t="inlineStr" s="0">
         <is>
-          <t>Row2_GearRod</t>
+          <t>GEAR_ROD_ROW2</t>
         </is>
       </c>
       <c r="G101" t="inlineStr" s="0">
@@ -6676,7 +6676,7 @@
       </c>
       <c r="F102" t="inlineStr" s="0">
         <is>
-          <t>Row2_GearRod</t>
+          <t>GEAR_ROD_ROW2</t>
         </is>
       </c>
       <c r="G102" t="inlineStr" s="0">
@@ -6743,7 +6743,7 @@
       </c>
       <c r="F103" t="inlineStr" s="0">
         <is>
-          <t>Row2_GearRod</t>
+          <t>GEAR_ROD_ROW2</t>
         </is>
       </c>
       <c r="G103" t="inlineStr" s="0">
@@ -6810,7 +6810,7 @@
       </c>
       <c r="F104" t="inlineStr" s="0">
         <is>
-          <t>Row2_GearStand_Left</t>
+          <t>STAND_ROW2_LEFT</t>
         </is>
       </c>
       <c r="G104" t="inlineStr" s="0">
@@ -6877,7 +6877,7 @@
       </c>
       <c r="F105" t="inlineStr" s="0">
         <is>
-          <t>Row2_GearStand_Left</t>
+          <t>STAND_ROW2_LEFT</t>
         </is>
       </c>
       <c r="G105" t="inlineStr" s="0">
@@ -6944,7 +6944,7 @@
       </c>
       <c r="F106" t="inlineStr" s="0">
         <is>
-          <t>Row2_GearStand_Left</t>
+          <t>STAND_ROW2_LEFT</t>
         </is>
       </c>
       <c r="G106" t="inlineStr" s="0">
@@ -7011,7 +7011,7 @@
       </c>
       <c r="F107" t="inlineStr" s="0">
         <is>
-          <t>Row2_GearStand_Left</t>
+          <t>STAND_ROW2_LEFT</t>
         </is>
       </c>
       <c r="G107" t="inlineStr" s="0">
@@ -7078,7 +7078,7 @@
       </c>
       <c r="F108" t="inlineStr" s="0">
         <is>
-          <t>Row2_GearStand_Left</t>
+          <t>STAND_ROW2_LEFT</t>
         </is>
       </c>
       <c r="G108" t="inlineStr" s="0">
@@ -7145,7 +7145,7 @@
       </c>
       <c r="F109" t="inlineStr" s="0">
         <is>
-          <t>Row2_GearStand_Left</t>
+          <t>STAND_ROW2_LEFT</t>
         </is>
       </c>
       <c r="G109" t="inlineStr" s="0">
@@ -7212,7 +7212,7 @@
       </c>
       <c r="F110" t="inlineStr" s="0">
         <is>
-          <t>Row2_GearStand_Left</t>
+          <t>STAND_ROW2_LEFT</t>
         </is>
       </c>
       <c r="G110" t="inlineStr" s="0">
@@ -7279,7 +7279,7 @@
       </c>
       <c r="F111" t="inlineStr" s="0">
         <is>
-          <t>Row2_GearStand_Left</t>
+          <t>STAND_ROW2_LEFT</t>
         </is>
       </c>
       <c r="G111" t="inlineStr" s="0">
@@ -7346,7 +7346,7 @@
       </c>
       <c r="F112" t="inlineStr" s="0">
         <is>
-          <t>Row2_GearStand_Left</t>
+          <t>STAND_ROW2_LEFT</t>
         </is>
       </c>
       <c r="G112" t="inlineStr" s="0">
@@ -7413,7 +7413,7 @@
       </c>
       <c r="F113" t="inlineStr" s="0">
         <is>
-          <t>Row2_GearStand_Left</t>
+          <t>STAND_ROW2_LEFT</t>
         </is>
       </c>
       <c r="G113" t="inlineStr" s="0">
@@ -7480,7 +7480,7 @@
       </c>
       <c r="F114" t="inlineStr" s="0">
         <is>
-          <t>Row2_GearStand_Left</t>
+          <t>STAND_ROW2_LEFT</t>
         </is>
       </c>
       <c r="G114" t="inlineStr" s="0">
@@ -7547,7 +7547,7 @@
       </c>
       <c r="F115" t="inlineStr" s="0">
         <is>
-          <t>Row2_GearStand_Left</t>
+          <t>STAND_ROW2_LEFT</t>
         </is>
       </c>
       <c r="G115" t="inlineStr" s="0">
@@ -7614,7 +7614,7 @@
       </c>
       <c r="F116" t="inlineStr" s="0">
         <is>
-          <t>Row2_GearStand_Right</t>
+          <t>STAND_ROW2_RIGHT</t>
         </is>
       </c>
       <c r="G116" t="inlineStr" s="0">
@@ -7681,7 +7681,7 @@
       </c>
       <c r="F117" t="inlineStr" s="0">
         <is>
-          <t>Row2_GearStand_Right</t>
+          <t>STAND_ROW2_RIGHT</t>
         </is>
       </c>
       <c r="G117" t="inlineStr" s="0">
@@ -7748,7 +7748,7 @@
       </c>
       <c r="F118" t="inlineStr" s="0">
         <is>
-          <t>Row2_GearStand_Right</t>
+          <t>STAND_ROW2_RIGHT</t>
         </is>
       </c>
       <c r="G118" t="inlineStr" s="0">
@@ -7815,7 +7815,7 @@
       </c>
       <c r="F119" t="inlineStr" s="0">
         <is>
-          <t>Row2_GearStand_Right</t>
+          <t>STAND_ROW2_RIGHT</t>
         </is>
       </c>
       <c r="G119" t="inlineStr" s="0">
@@ -7882,7 +7882,7 @@
       </c>
       <c r="F120" t="inlineStr" s="0">
         <is>
-          <t>Row2_GearStand_Right</t>
+          <t>STAND_ROW2_RIGHT</t>
         </is>
       </c>
       <c r="G120" t="inlineStr" s="0">
@@ -7949,7 +7949,7 @@
       </c>
       <c r="F121" t="inlineStr" s="0">
         <is>
-          <t>Row2_GearStand_Right</t>
+          <t>STAND_ROW2_RIGHT</t>
         </is>
       </c>
       <c r="G121" t="inlineStr" s="0">
@@ -8016,7 +8016,7 @@
       </c>
       <c r="F122" t="inlineStr" s="0">
         <is>
-          <t>Row2_GearStand_Right</t>
+          <t>STAND_ROW2_RIGHT</t>
         </is>
       </c>
       <c r="G122" t="inlineStr" s="0">
@@ -8083,7 +8083,7 @@
       </c>
       <c r="F123" t="inlineStr" s="0">
         <is>
-          <t>Row2_GearStand_Right</t>
+          <t>STAND_ROW2_RIGHT</t>
         </is>
       </c>
       <c r="G123" t="inlineStr" s="0">
@@ -8150,7 +8150,7 @@
       </c>
       <c r="F124" t="inlineStr" s="0">
         <is>
-          <t>Row2_GearStand_Right</t>
+          <t>STAND_ROW2_RIGHT</t>
         </is>
       </c>
       <c r="G124" t="inlineStr" s="0">
@@ -8217,7 +8217,7 @@
       </c>
       <c r="F125" t="inlineStr" s="0">
         <is>
-          <t>Row2_GearStand_Right</t>
+          <t>STAND_ROW2_RIGHT</t>
         </is>
       </c>
       <c r="G125" t="inlineStr" s="0">
@@ -8284,7 +8284,7 @@
       </c>
       <c r="F126" t="inlineStr" s="0">
         <is>
-          <t>Row2_GearStand_Right</t>
+          <t>STAND_ROW2_RIGHT</t>
         </is>
       </c>
       <c r="G126" t="inlineStr" s="0">
@@ -8351,7 +8351,7 @@
       </c>
       <c r="F127" t="inlineStr" s="0">
         <is>
-          <t>Row2_GearStand_Right</t>
+          <t>STAND_ROW2_RIGHT</t>
         </is>
       </c>
       <c r="G127" t="inlineStr" s="0">
@@ -8418,7 +8418,7 @@
       </c>
       <c r="F128" t="inlineStr" s="0">
         <is>
-          <t>Row2_Gear_Left</t>
+          <t>GEAR_ROW2_LEFT</t>
         </is>
       </c>
       <c r="G128" t="inlineStr" s="0">
@@ -8485,7 +8485,7 @@
       </c>
       <c r="F129" t="inlineStr" s="0">
         <is>
-          <t>Row2_Gear_Left</t>
+          <t>GEAR_ROW2_LEFT</t>
         </is>
       </c>
       <c r="G129" t="inlineStr" s="0">
@@ -8552,7 +8552,7 @@
       </c>
       <c r="F130" t="inlineStr" s="0">
         <is>
-          <t>Row2_Gear_Left</t>
+          <t>GEAR_ROW2_LEFT</t>
         </is>
       </c>
       <c r="G130" t="inlineStr" s="0">
@@ -8619,7 +8619,7 @@
       </c>
       <c r="F131" t="inlineStr" s="0">
         <is>
-          <t>Row2_Gear_Left</t>
+          <t>GEAR_ROW2_LEFT</t>
         </is>
       </c>
       <c r="G131" t="inlineStr" s="0">
@@ -8686,7 +8686,7 @@
       </c>
       <c r="F132" t="inlineStr" s="0">
         <is>
-          <t>Row2_Gear_Left</t>
+          <t>GEAR_ROW2_LEFT</t>
         </is>
       </c>
       <c r="G132" t="inlineStr" s="0">
@@ -8753,7 +8753,7 @@
       </c>
       <c r="F133" t="inlineStr" s="0">
         <is>
-          <t>Row2_Gear_Left</t>
+          <t>GEAR_ROW2_LEFT</t>
         </is>
       </c>
       <c r="G133" t="inlineStr" s="0">
@@ -8820,7 +8820,7 @@
       </c>
       <c r="F134" t="inlineStr" s="0">
         <is>
-          <t>Row2_Gear_Left</t>
+          <t>GEAR_ROW2_LEFT</t>
         </is>
       </c>
       <c r="G134" t="inlineStr" s="0">
@@ -8887,7 +8887,7 @@
       </c>
       <c r="F135" t="inlineStr" s="0">
         <is>
-          <t>Row2_Gear_Left</t>
+          <t>GEAR_ROW2_LEFT</t>
         </is>
       </c>
       <c r="G135" t="inlineStr" s="0">
@@ -8954,7 +8954,7 @@
       </c>
       <c r="F136" t="inlineStr" s="0">
         <is>
-          <t>Row2_Gear_Left</t>
+          <t>GEAR_ROW2_LEFT</t>
         </is>
       </c>
       <c r="G136" t="inlineStr" s="0">
@@ -9021,7 +9021,7 @@
       </c>
       <c r="F137" t="inlineStr" s="0">
         <is>
-          <t>Row2_Gear_Left</t>
+          <t>GEAR_ROW2_LEFT</t>
         </is>
       </c>
       <c r="G137" t="inlineStr" s="0">
@@ -9088,7 +9088,7 @@
       </c>
       <c r="F138" t="inlineStr" s="0">
         <is>
-          <t>Row2_Gear_Left</t>
+          <t>GEAR_ROW2_LEFT</t>
         </is>
       </c>
       <c r="G138" t="inlineStr" s="0">
@@ -9155,7 +9155,7 @@
       </c>
       <c r="F139" t="inlineStr" s="0">
         <is>
-          <t>Row2_Gear_Right</t>
+          <t>GEAR_ROW2_RIGHT</t>
         </is>
       </c>
       <c r="G139" t="inlineStr" s="0">
@@ -9222,7 +9222,7 @@
       </c>
       <c r="F140" t="inlineStr" s="0">
         <is>
-          <t>Row2_Gear_Right</t>
+          <t>GEAR_ROW2_RIGHT</t>
         </is>
       </c>
       <c r="G140" t="inlineStr" s="0">
@@ -9289,7 +9289,7 @@
       </c>
       <c r="F141" t="inlineStr" s="0">
         <is>
-          <t>Row2_Gear_Right</t>
+          <t>GEAR_ROW2_RIGHT</t>
         </is>
       </c>
       <c r="G141" t="inlineStr" s="0">
@@ -9356,7 +9356,7 @@
       </c>
       <c r="F142" t="inlineStr" s="0">
         <is>
-          <t>Row2_Gear_Right</t>
+          <t>GEAR_ROW2_RIGHT</t>
         </is>
       </c>
       <c r="G142" t="inlineStr" s="0">
@@ -9423,7 +9423,7 @@
       </c>
       <c r="F143" t="inlineStr" s="0">
         <is>
-          <t>Row2_Gear_Right</t>
+          <t>GEAR_ROW2_RIGHT</t>
         </is>
       </c>
       <c r="G143" t="inlineStr" s="0">
@@ -9490,7 +9490,7 @@
       </c>
       <c r="F144" t="inlineStr" s="0">
         <is>
-          <t>Row2_Gear_Right</t>
+          <t>GEAR_ROW2_RIGHT</t>
         </is>
       </c>
       <c r="G144" t="inlineStr" s="0">
@@ -9557,7 +9557,7 @@
       </c>
       <c r="F145" t="inlineStr" s="0">
         <is>
-          <t>Row2_Gear_Right</t>
+          <t>GEAR_ROW2_RIGHT</t>
         </is>
       </c>
       <c r="G145" t="inlineStr" s="0">
@@ -9624,7 +9624,7 @@
       </c>
       <c r="F146" t="inlineStr" s="0">
         <is>
-          <t>Row2_Gear_Right</t>
+          <t>GEAR_ROW2_RIGHT</t>
         </is>
       </c>
       <c r="G146" t="inlineStr" s="0">
@@ -9691,7 +9691,7 @@
       </c>
       <c r="F147" t="inlineStr" s="0">
         <is>
-          <t>Row2_Gear_Right</t>
+          <t>GEAR_ROW2_RIGHT</t>
         </is>
       </c>
       <c r="G147" t="inlineStr" s="0">
@@ -9758,7 +9758,7 @@
       </c>
       <c r="F148" t="inlineStr" s="0">
         <is>
-          <t>Row2_Gear_Right</t>
+          <t>GEAR_ROW2_RIGHT</t>
         </is>
       </c>
       <c r="G148" t="inlineStr" s="0">
@@ -9825,7 +9825,7 @@
       </c>
       <c r="F149" t="inlineStr" s="0">
         <is>
-          <t>Row2_Gear_Right</t>
+          <t>GEAR_ROW2_RIGHT</t>
         </is>
       </c>
       <c r="G149" t="inlineStr" s="0">
@@ -9892,7 +9892,7 @@
       </c>
       <c r="F150" t="inlineStr" s="0">
         <is>
-          <t>Row2_Screws</t>
+          <t>SCREW_ROW2</t>
         </is>
       </c>
       <c r="G150" t="inlineStr" s="0">
@@ -9959,7 +9959,7 @@
       </c>
       <c r="F151" t="inlineStr" s="0">
         <is>
-          <t>Row2_Screws</t>
+          <t>SCREW_ROW2</t>
         </is>
       </c>
       <c r="G151" t="inlineStr" s="0">
@@ -10026,7 +10026,7 @@
       </c>
       <c r="F152" t="inlineStr" s="0">
         <is>
-          <t>Row2_Screws</t>
+          <t>SCREW_ROW2</t>
         </is>
       </c>
       <c r="G152" t="inlineStr" s="0">
@@ -10093,7 +10093,7 @@
       </c>
       <c r="F153" t="inlineStr" s="0">
         <is>
-          <t>Row2_Screws</t>
+          <t>SCREW_ROW2</t>
         </is>
       </c>
       <c r="G153" t="inlineStr" s="0">
@@ -10160,7 +10160,7 @@
       </c>
       <c r="F154" t="inlineStr" s="0">
         <is>
-          <t>Row2_Screws</t>
+          <t>SCREW_ROW2</t>
         </is>
       </c>
       <c r="G154" t="inlineStr" s="0">
@@ -10227,7 +10227,7 @@
       </c>
       <c r="F155" t="inlineStr" s="0">
         <is>
-          <t>Row2_Screws</t>
+          <t>SCREW_ROW2</t>
         </is>
       </c>
       <c r="G155" t="inlineStr" s="0">
@@ -10294,7 +10294,7 @@
       </c>
       <c r="F156" t="inlineStr" s="0">
         <is>
-          <t>Row2_Screws</t>
+          <t>SCREW_ROW2</t>
         </is>
       </c>
       <c r="G156" t="inlineStr" s="0">
@@ -10361,7 +10361,7 @@
       </c>
       <c r="F157" t="inlineStr" s="0">
         <is>
-          <t>Row2_Screws</t>
+          <t>SCREW_ROW2</t>
         </is>
       </c>
       <c r="G157" t="inlineStr" s="0">
@@ -10428,7 +10428,7 @@
       </c>
       <c r="F158" t="inlineStr" s="0">
         <is>
-          <t>Row2_Screws</t>
+          <t>SCREW_ROW2</t>
         </is>
       </c>
       <c r="G158" t="inlineStr" s="0">
@@ -10495,7 +10495,7 @@
       </c>
       <c r="F159" t="inlineStr" s="0">
         <is>
-          <t>Row3_GearRod</t>
+          <t>GEAR_ROD_ROW3</t>
         </is>
       </c>
       <c r="G159" t="inlineStr" s="0">
@@ -10562,7 +10562,7 @@
       </c>
       <c r="F160" t="inlineStr" s="0">
         <is>
-          <t>Row3_GearRod</t>
+          <t>GEAR_ROD_ROW3</t>
         </is>
       </c>
       <c r="G160" t="inlineStr" s="0">
@@ -10629,7 +10629,7 @@
       </c>
       <c r="F161" t="inlineStr" s="0">
         <is>
-          <t>Row3_GearRod</t>
+          <t>GEAR_ROD_ROW3</t>
         </is>
       </c>
       <c r="G161" t="inlineStr" s="0">
@@ -10696,7 +10696,7 @@
       </c>
       <c r="F162" t="inlineStr" s="0">
         <is>
-          <t>Row3_GearRod</t>
+          <t>GEAR_ROD_ROW3</t>
         </is>
       </c>
       <c r="G162" t="inlineStr" s="0">
@@ -10763,7 +10763,7 @@
       </c>
       <c r="F163" t="inlineStr" s="0">
         <is>
-          <t>Row3_GearRod</t>
+          <t>GEAR_ROD_ROW3</t>
         </is>
       </c>
       <c r="G163" t="inlineStr" s="0">
@@ -10830,7 +10830,7 @@
       </c>
       <c r="F164" t="inlineStr" s="0">
         <is>
-          <t>Row3_GearRod</t>
+          <t>GEAR_ROD_ROW3</t>
         </is>
       </c>
       <c r="G164" t="inlineStr" s="0">
@@ -10897,7 +10897,7 @@
       </c>
       <c r="F165" t="inlineStr" s="0">
         <is>
-          <t>Row3_GearRod</t>
+          <t>GEAR_ROD_ROW3</t>
         </is>
       </c>
       <c r="G165" t="inlineStr" s="0">
@@ -10964,7 +10964,7 @@
       </c>
       <c r="F166" t="inlineStr" s="0">
         <is>
-          <t>Row3_GearRod</t>
+          <t>GEAR_ROD_ROW3</t>
         </is>
       </c>
       <c r="G166" t="inlineStr" s="0">
@@ -11031,7 +11031,7 @@
       </c>
       <c r="F167" t="inlineStr" s="0">
         <is>
-          <t>Row3_GearRod</t>
+          <t>GEAR_ROD_ROW3</t>
         </is>
       </c>
       <c r="G167" t="inlineStr" s="0">
@@ -11098,7 +11098,7 @@
       </c>
       <c r="F168" t="inlineStr" s="0">
         <is>
-          <t>Row3_GearRod</t>
+          <t>GEAR_ROD_ROW3</t>
         </is>
       </c>
       <c r="G168" t="inlineStr" s="0">
@@ -11165,7 +11165,7 @@
       </c>
       <c r="F169" t="inlineStr" s="0">
         <is>
-          <t>Row3_GearRod</t>
+          <t>GEAR_ROD_ROW3</t>
         </is>
       </c>
       <c r="G169" t="inlineStr" s="0">
@@ -11232,7 +11232,7 @@
       </c>
       <c r="F170" t="inlineStr" s="0">
         <is>
-          <t>Row3_GearRod</t>
+          <t>GEAR_ROD_ROW3</t>
         </is>
       </c>
       <c r="G170" t="inlineStr" s="0">
@@ -11299,7 +11299,7 @@
       </c>
       <c r="F171" t="inlineStr" s="0">
         <is>
-          <t>Row3_GearStand_Left</t>
+          <t>STAND_ROW3_LEFT</t>
         </is>
       </c>
       <c r="G171" t="inlineStr" s="0">
@@ -11366,7 +11366,7 @@
       </c>
       <c r="F172" t="inlineStr" s="0">
         <is>
-          <t>Row3_GearStand_Left</t>
+          <t>STAND_ROW3_LEFT</t>
         </is>
       </c>
       <c r="G172" t="inlineStr" s="0">
@@ -11433,7 +11433,7 @@
       </c>
       <c r="F173" t="inlineStr" s="0">
         <is>
-          <t>Row3_GearStand_Left</t>
+          <t>STAND_ROW3_LEFT</t>
         </is>
       </c>
       <c r="G173" t="inlineStr" s="0">
@@ -11500,7 +11500,7 @@
       </c>
       <c r="F174" t="inlineStr" s="0">
         <is>
-          <t>Row3_GearStand_Left</t>
+          <t>STAND_ROW3_LEFT</t>
         </is>
       </c>
       <c r="G174" t="inlineStr" s="0">
@@ -11567,7 +11567,7 @@
       </c>
       <c r="F175" t="inlineStr" s="0">
         <is>
-          <t>Row3_GearStand_Left</t>
+          <t>STAND_ROW3_LEFT</t>
         </is>
       </c>
       <c r="G175" t="inlineStr" s="0">
@@ -11634,7 +11634,7 @@
       </c>
       <c r="F176" t="inlineStr" s="0">
         <is>
-          <t>Row3_GearStand_Left</t>
+          <t>STAND_ROW3_LEFT</t>
         </is>
       </c>
       <c r="G176" t="inlineStr" s="0">
@@ -11701,7 +11701,7 @@
       </c>
       <c r="F177" t="inlineStr" s="0">
         <is>
-          <t>Row3_GearStand_Left</t>
+          <t>STAND_ROW3_LEFT</t>
         </is>
       </c>
       <c r="G177" t="inlineStr" s="0">
@@ -11768,7 +11768,7 @@
       </c>
       <c r="F178" t="inlineStr" s="0">
         <is>
-          <t>Row3_GearStand_Left</t>
+          <t>STAND_ROW3_LEFT</t>
         </is>
       </c>
       <c r="G178" t="inlineStr" s="0">
@@ -11835,7 +11835,7 @@
       </c>
       <c r="F179" t="inlineStr" s="0">
         <is>
-          <t>Row3_GearStand_Left</t>
+          <t>STAND_ROW3_LEFT</t>
         </is>
       </c>
       <c r="G179" t="inlineStr" s="0">
@@ -11902,7 +11902,7 @@
       </c>
       <c r="F180" t="inlineStr" s="0">
         <is>
-          <t>Row3_GearStand_Left</t>
+          <t>STAND_ROW3_LEFT</t>
         </is>
       </c>
       <c r="G180" t="inlineStr" s="0">
@@ -11969,7 +11969,7 @@
       </c>
       <c r="F181" t="inlineStr" s="0">
         <is>
-          <t>Row3_GearStand_Left</t>
+          <t>STAND_ROW3_LEFT</t>
         </is>
       </c>
       <c r="G181" t="inlineStr" s="0">
@@ -12036,7 +12036,7 @@
       </c>
       <c r="F182" t="inlineStr" s="0">
         <is>
-          <t>Row3_GearStand_Left</t>
+          <t>STAND_ROW3_LEFT</t>
         </is>
       </c>
       <c r="G182" t="inlineStr" s="0">
@@ -12103,7 +12103,7 @@
       </c>
       <c r="F183" t="inlineStr" s="0">
         <is>
-          <t>Row3_GearStand_Right</t>
+          <t>STAND_ROW3_RIGHT</t>
         </is>
       </c>
       <c r="G183" t="inlineStr" s="0">
@@ -12170,7 +12170,7 @@
       </c>
       <c r="F184" t="inlineStr" s="0">
         <is>
-          <t>Row3_GearStand_Right</t>
+          <t>STAND_ROW3_RIGHT</t>
         </is>
       </c>
       <c r="G184" t="inlineStr" s="0">
@@ -12237,7 +12237,7 @@
       </c>
       <c r="F185" t="inlineStr" s="0">
         <is>
-          <t>Row3_GearStand_Right</t>
+          <t>STAND_ROW3_RIGHT</t>
         </is>
       </c>
       <c r="G185" t="inlineStr" s="0">
@@ -12304,7 +12304,7 @@
       </c>
       <c r="F186" t="inlineStr" s="0">
         <is>
-          <t>Row3_GearStand_Right</t>
+          <t>STAND_ROW3_RIGHT</t>
         </is>
       </c>
       <c r="G186" t="inlineStr" s="0">
@@ -12371,7 +12371,7 @@
       </c>
       <c r="F187" t="inlineStr" s="0">
         <is>
-          <t>Row3_GearStand_Right</t>
+          <t>STAND_ROW3_RIGHT</t>
         </is>
       </c>
       <c r="G187" t="inlineStr" s="0">
@@ -12438,7 +12438,7 @@
       </c>
       <c r="F188" t="inlineStr" s="0">
         <is>
-          <t>Row3_GearStand_Right</t>
+          <t>STAND_ROW3_RIGHT</t>
         </is>
       </c>
       <c r="G188" t="inlineStr" s="0">
@@ -12505,7 +12505,7 @@
       </c>
       <c r="F189" t="inlineStr" s="0">
         <is>
-          <t>Row3_GearStand_Right</t>
+          <t>STAND_ROW3_RIGHT</t>
         </is>
       </c>
       <c r="G189" t="inlineStr" s="0">
@@ -12572,7 +12572,7 @@
       </c>
       <c r="F190" t="inlineStr" s="0">
         <is>
-          <t>Row3_GearStand_Right</t>
+          <t>STAND_ROW3_RIGHT</t>
         </is>
       </c>
       <c r="G190" t="inlineStr" s="0">
@@ -12639,7 +12639,7 @@
       </c>
       <c r="F191" t="inlineStr" s="0">
         <is>
-          <t>Row3_GearStand_Right</t>
+          <t>STAND_ROW3_RIGHT</t>
         </is>
       </c>
       <c r="G191" t="inlineStr" s="0">
@@ -12706,7 +12706,7 @@
       </c>
       <c r="F192" t="inlineStr" s="0">
         <is>
-          <t>Row3_GearStand_Right</t>
+          <t>STAND_ROW3_RIGHT</t>
         </is>
       </c>
       <c r="G192" t="inlineStr" s="0">
@@ -12773,7 +12773,7 @@
       </c>
       <c r="F193" t="inlineStr" s="0">
         <is>
-          <t>Row3_GearStand_Right</t>
+          <t>STAND_ROW3_RIGHT</t>
         </is>
       </c>
       <c r="G193" t="inlineStr" s="0">
@@ -12840,7 +12840,7 @@
       </c>
       <c r="F194" t="inlineStr" s="0">
         <is>
-          <t>Row3_GearStand_Right</t>
+          <t>STAND_ROW3_RIGHT</t>
         </is>
       </c>
       <c r="G194" t="inlineStr" s="0">
@@ -12907,7 +12907,7 @@
       </c>
       <c r="F195" t="inlineStr" s="0">
         <is>
-          <t>Row3_Gear_Left</t>
+          <t>GEAR_ROW3_LEFT</t>
         </is>
       </c>
       <c r="G195" t="inlineStr" s="0">
@@ -12974,7 +12974,7 @@
       </c>
       <c r="F196" t="inlineStr" s="0">
         <is>
-          <t>Row3_Gear_Left</t>
+          <t>GEAR_ROW3_LEFT</t>
         </is>
       </c>
       <c r="G196" t="inlineStr" s="0">
@@ -13041,7 +13041,7 @@
       </c>
       <c r="F197" t="inlineStr" s="0">
         <is>
-          <t>Row3_Gear_Left</t>
+          <t>GEAR_ROW3_LEFT</t>
         </is>
       </c>
       <c r="G197" t="inlineStr" s="0">
@@ -13108,7 +13108,7 @@
       </c>
       <c r="F198" t="inlineStr" s="0">
         <is>
-          <t>Row3_Gear_Left</t>
+          <t>GEAR_ROW3_LEFT</t>
         </is>
       </c>
       <c r="G198" t="inlineStr" s="0">
@@ -13175,7 +13175,7 @@
       </c>
       <c r="F199" t="inlineStr" s="0">
         <is>
-          <t>Row3_Gear_Left</t>
+          <t>GEAR_ROW3_LEFT</t>
         </is>
       </c>
       <c r="G199" t="inlineStr" s="0">
@@ -13242,7 +13242,7 @@
       </c>
       <c r="F200" t="inlineStr" s="0">
         <is>
-          <t>Row3_Gear_Left</t>
+          <t>GEAR_ROW3_LEFT</t>
         </is>
       </c>
       <c r="G200" t="inlineStr" s="0">
@@ -13309,7 +13309,7 @@
       </c>
       <c r="F201" t="inlineStr" s="0">
         <is>
-          <t>Row3_Gear_Left</t>
+          <t>GEAR_ROW3_LEFT</t>
         </is>
       </c>
       <c r="G201" t="inlineStr" s="0">
@@ -13376,7 +13376,7 @@
       </c>
       <c r="F202" t="inlineStr" s="0">
         <is>
-          <t>Row3_Gear_Left</t>
+          <t>GEAR_ROW3_LEFT</t>
         </is>
       </c>
       <c r="G202" t="inlineStr" s="0">
@@ -13443,7 +13443,7 @@
       </c>
       <c r="F203" t="inlineStr" s="0">
         <is>
-          <t>Row3_Gear_Left</t>
+          <t>GEAR_ROW3_LEFT</t>
         </is>
       </c>
       <c r="G203" t="inlineStr" s="0">
@@ -13510,7 +13510,7 @@
       </c>
       <c r="F204" t="inlineStr" s="0">
         <is>
-          <t>Row3_Gear_Left</t>
+          <t>GEAR_ROW3_LEFT</t>
         </is>
       </c>
       <c r="G204" t="inlineStr" s="0">
@@ -13577,7 +13577,7 @@
       </c>
       <c r="F205" t="inlineStr" s="0">
         <is>
-          <t>Row3_Gear_Left</t>
+          <t>GEAR_ROW3_LEFT</t>
         </is>
       </c>
       <c r="G205" t="inlineStr" s="0">
@@ -13644,7 +13644,7 @@
       </c>
       <c r="F206" t="inlineStr" s="0">
         <is>
-          <t>Row3_Gear_Right</t>
+          <t>GEAR_ROW3_RIGHT</t>
         </is>
       </c>
       <c r="G206" t="inlineStr" s="0">
@@ -13711,7 +13711,7 @@
       </c>
       <c r="F207" t="inlineStr" s="0">
         <is>
-          <t>Row3_Gear_Right</t>
+          <t>GEAR_ROW3_RIGHT</t>
         </is>
       </c>
       <c r="G207" t="inlineStr" s="0">
@@ -13778,7 +13778,7 @@
       </c>
       <c r="F208" t="inlineStr" s="0">
         <is>
-          <t>Row3_Gear_Right</t>
+          <t>GEAR_ROW3_RIGHT</t>
         </is>
       </c>
       <c r="G208" t="inlineStr" s="0">
@@ -13845,7 +13845,7 @@
       </c>
       <c r="F209" t="inlineStr" s="0">
         <is>
-          <t>Row3_Gear_Right</t>
+          <t>GEAR_ROW3_RIGHT</t>
         </is>
       </c>
       <c r="G209" t="inlineStr" s="0">
@@ -13912,7 +13912,7 @@
       </c>
       <c r="F210" t="inlineStr" s="0">
         <is>
-          <t>Row3_Gear_Right</t>
+          <t>GEAR_ROW3_RIGHT</t>
         </is>
       </c>
       <c r="G210" t="inlineStr" s="0">
@@ -13979,7 +13979,7 @@
       </c>
       <c r="F211" t="inlineStr" s="0">
         <is>
-          <t>Row3_Gear_Right</t>
+          <t>GEAR_ROW3_RIGHT</t>
         </is>
       </c>
       <c r="G211" t="inlineStr" s="0">
@@ -14046,7 +14046,7 @@
       </c>
       <c r="F212" t="inlineStr" s="0">
         <is>
-          <t>Row3_Gear_Right</t>
+          <t>GEAR_ROW3_RIGHT</t>
         </is>
       </c>
       <c r="G212" t="inlineStr" s="0">
@@ -14113,7 +14113,7 @@
       </c>
       <c r="F213" t="inlineStr" s="0">
         <is>
-          <t>Row3_Gear_Right</t>
+          <t>GEAR_ROW3_RIGHT</t>
         </is>
       </c>
       <c r="G213" t="inlineStr" s="0">
@@ -14180,7 +14180,7 @@
       </c>
       <c r="F214" t="inlineStr" s="0">
         <is>
-          <t>Row3_Gear_Right</t>
+          <t>GEAR_ROW3_RIGHT</t>
         </is>
       </c>
       <c r="G214" t="inlineStr" s="0">
@@ -14247,7 +14247,7 @@
       </c>
       <c r="F215" t="inlineStr" s="0">
         <is>
-          <t>Row3_Gear_Right</t>
+          <t>GEAR_ROW3_RIGHT</t>
         </is>
       </c>
       <c r="G215" t="inlineStr" s="0">
@@ -14314,7 +14314,7 @@
       </c>
       <c r="F216" t="inlineStr" s="0">
         <is>
-          <t>Row3_Gear_Right</t>
+          <t>GEAR_ROW3_RIGHT</t>
         </is>
       </c>
       <c r="G216" t="inlineStr" s="0">
@@ -14381,7 +14381,7 @@
       </c>
       <c r="F217" t="inlineStr" s="0">
         <is>
-          <t>Row3_Screws</t>
+          <t>SCREW_ROW3</t>
         </is>
       </c>
       <c r="G217" t="inlineStr" s="0">
@@ -14448,7 +14448,7 @@
       </c>
       <c r="F218" t="inlineStr" s="0">
         <is>
-          <t>Row3_Screws</t>
+          <t>SCREW_ROW3</t>
         </is>
       </c>
       <c r="G218" t="inlineStr" s="0">
@@ -14515,7 +14515,7 @@
       </c>
       <c r="F219" t="inlineStr" s="0">
         <is>
-          <t>Row3_Screws</t>
+          <t>SCREW_ROW3</t>
         </is>
       </c>
       <c r="G219" t="inlineStr" s="0">
@@ -14582,7 +14582,7 @@
       </c>
       <c r="F220" t="inlineStr" s="0">
         <is>
-          <t>Row3_Screws</t>
+          <t>SCREW_ROW3</t>
         </is>
       </c>
       <c r="G220" t="inlineStr" s="0">
@@ -14649,7 +14649,7 @@
       </c>
       <c r="F221" t="inlineStr" s="0">
         <is>
-          <t>Row3_Screws</t>
+          <t>SCREW_ROW3</t>
         </is>
       </c>
       <c r="G221" t="inlineStr" s="0">
@@ -14716,7 +14716,7 @@
       </c>
       <c r="F222" t="inlineStr" s="0">
         <is>
-          <t>Row3_Screws</t>
+          <t>SCREW_ROW3</t>
         </is>
       </c>
       <c r="G222" t="inlineStr" s="0">
@@ -14783,7 +14783,7 @@
       </c>
       <c r="F223" t="inlineStr" s="0">
         <is>
-          <t>Row3_Screws</t>
+          <t>SCREW_ROW3</t>
         </is>
       </c>
       <c r="G223" t="inlineStr" s="0">
@@ -14850,7 +14850,7 @@
       </c>
       <c r="F224" t="inlineStr" s="0">
         <is>
-          <t>Row3_Screws</t>
+          <t>SCREW_ROW3</t>
         </is>
       </c>
       <c r="G224" t="inlineStr" s="0">
@@ -14917,7 +14917,7 @@
       </c>
       <c r="F225" t="inlineStr" s="0">
         <is>
-          <t>Row3_Screws</t>
+          <t>SCREW_ROW3</t>
         </is>
       </c>
       <c r="G225" t="inlineStr" s="0">
@@ -14984,7 +14984,7 @@
       </c>
       <c r="F226" t="inlineStr" s="0">
         <is>
-          <t>Row4_GearRod</t>
+          <t>GEAR_ROD_ROW4</t>
         </is>
       </c>
       <c r="G226" t="inlineStr" s="0">
@@ -15051,7 +15051,7 @@
       </c>
       <c r="F227" t="inlineStr" s="0">
         <is>
-          <t>Row4_GearRod</t>
+          <t>GEAR_ROD_ROW4</t>
         </is>
       </c>
       <c r="G227" t="inlineStr" s="0">
@@ -15118,7 +15118,7 @@
       </c>
       <c r="F228" t="inlineStr" s="0">
         <is>
-          <t>Row4_GearRod</t>
+          <t>GEAR_ROD_ROW4</t>
         </is>
       </c>
       <c r="G228" t="inlineStr" s="0">
@@ -15185,7 +15185,7 @@
       </c>
       <c r="F229" t="inlineStr" s="0">
         <is>
-          <t>Row4_GearRod</t>
+          <t>GEAR_ROD_ROW4</t>
         </is>
       </c>
       <c r="G229" t="inlineStr" s="0">
@@ -15252,7 +15252,7 @@
       </c>
       <c r="F230" t="inlineStr" s="0">
         <is>
-          <t>Row4_GearRod</t>
+          <t>GEAR_ROD_ROW4</t>
         </is>
       </c>
       <c r="G230" t="inlineStr" s="0">
@@ -15319,7 +15319,7 @@
       </c>
       <c r="F231" t="inlineStr" s="0">
         <is>
-          <t>Row4_GearRod</t>
+          <t>GEAR_ROD_ROW4</t>
         </is>
       </c>
       <c r="G231" t="inlineStr" s="0">
@@ -15386,7 +15386,7 @@
       </c>
       <c r="F232" t="inlineStr" s="0">
         <is>
-          <t>Row4_GearRod</t>
+          <t>GEAR_ROD_ROW4</t>
         </is>
       </c>
       <c r="G232" t="inlineStr" s="0">
@@ -15453,7 +15453,7 @@
       </c>
       <c r="F233" t="inlineStr" s="0">
         <is>
-          <t>Row4_GearRod</t>
+          <t>GEAR_ROD_ROW4</t>
         </is>
       </c>
       <c r="G233" t="inlineStr" s="0">
@@ -15520,7 +15520,7 @@
       </c>
       <c r="F234" t="inlineStr" s="0">
         <is>
-          <t>Row4_GearRod</t>
+          <t>GEAR_ROD_ROW4</t>
         </is>
       </c>
       <c r="G234" t="inlineStr" s="0">
@@ -15587,7 +15587,7 @@
       </c>
       <c r="F235" t="inlineStr" s="0">
         <is>
-          <t>Row4_GearRod</t>
+          <t>GEAR_ROD_ROW4</t>
         </is>
       </c>
       <c r="G235" t="inlineStr" s="0">
@@ -15654,7 +15654,7 @@
       </c>
       <c r="F236" t="inlineStr" s="0">
         <is>
-          <t>Row4_GearRod</t>
+          <t>GEAR_ROD_ROW4</t>
         </is>
       </c>
       <c r="G236" t="inlineStr" s="0">
@@ -15721,7 +15721,7 @@
       </c>
       <c r="F237" t="inlineStr" s="0">
         <is>
-          <t>Row4_GearRod</t>
+          <t>GEAR_ROD_ROW4</t>
         </is>
       </c>
       <c r="G237" t="inlineStr" s="0">
@@ -15788,7 +15788,7 @@
       </c>
       <c r="F238" t="inlineStr" s="0">
         <is>
-          <t>Row4_GearStand_Left</t>
+          <t>STAND_ROW4_LEFT</t>
         </is>
       </c>
       <c r="G238" t="inlineStr" s="0">
@@ -15855,7 +15855,7 @@
       </c>
       <c r="F239" t="inlineStr" s="0">
         <is>
-          <t>Row4_GearStand_Left</t>
+          <t>STAND_ROW4_LEFT</t>
         </is>
       </c>
       <c r="G239" t="inlineStr" s="0">
@@ -15922,7 +15922,7 @@
       </c>
       <c r="F240" t="inlineStr" s="0">
         <is>
-          <t>Row4_GearStand_Left</t>
+          <t>STAND_ROW4_LEFT</t>
         </is>
       </c>
       <c r="G240" t="inlineStr" s="0">
@@ -15989,7 +15989,7 @@
       </c>
       <c r="F241" t="inlineStr" s="0">
         <is>
-          <t>Row4_GearStand_Left</t>
+          <t>STAND_ROW4_LEFT</t>
         </is>
       </c>
       <c r="G241" t="inlineStr" s="0">
@@ -16056,7 +16056,7 @@
       </c>
       <c r="F242" t="inlineStr" s="0">
         <is>
-          <t>Row4_GearStand_Left</t>
+          <t>STAND_ROW4_LEFT</t>
         </is>
       </c>
       <c r="G242" t="inlineStr" s="0">
@@ -16123,7 +16123,7 @@
       </c>
       <c r="F243" t="inlineStr" s="0">
         <is>
-          <t>Row4_GearStand_Left</t>
+          <t>STAND_ROW4_LEFT</t>
         </is>
       </c>
       <c r="G243" t="inlineStr" s="0">
@@ -16190,7 +16190,7 @@
       </c>
       <c r="F244" t="inlineStr" s="0">
         <is>
-          <t>Row4_GearStand_Left</t>
+          <t>STAND_ROW4_LEFT</t>
         </is>
       </c>
       <c r="G244" t="inlineStr" s="0">
@@ -16257,7 +16257,7 @@
       </c>
       <c r="F245" t="inlineStr" s="0">
         <is>
-          <t>Row4_GearStand_Left</t>
+          <t>STAND_ROW4_LEFT</t>
         </is>
       </c>
       <c r="G245" t="inlineStr" s="0">
@@ -16324,7 +16324,7 @@
       </c>
       <c r="F246" t="inlineStr" s="0">
         <is>
-          <t>Row4_GearStand_Left</t>
+          <t>STAND_ROW4_LEFT</t>
         </is>
       </c>
       <c r="G246" t="inlineStr" s="0">
@@ -16391,7 +16391,7 @@
       </c>
       <c r="F247" t="inlineStr" s="0">
         <is>
-          <t>Row4_GearStand_Left</t>
+          <t>STAND_ROW4_LEFT</t>
         </is>
       </c>
       <c r="G247" t="inlineStr" s="0">
@@ -16458,7 +16458,7 @@
       </c>
       <c r="F248" t="inlineStr" s="0">
         <is>
-          <t>Row4_GearStand_Left</t>
+          <t>STAND_ROW4_LEFT</t>
         </is>
       </c>
       <c r="G248" t="inlineStr" s="0">
@@ -16525,7 +16525,7 @@
       </c>
       <c r="F249" t="inlineStr" s="0">
         <is>
-          <t>Row4_GearStand_Left</t>
+          <t>STAND_ROW4_LEFT</t>
         </is>
       </c>
       <c r="G249" t="inlineStr" s="0">
@@ -16592,7 +16592,7 @@
       </c>
       <c r="F250" t="inlineStr" s="0">
         <is>
-          <t>Row4_GearStand_Right</t>
+          <t>STAND_ROW4_RIGHT</t>
         </is>
       </c>
       <c r="G250" t="inlineStr" s="0">
@@ -16659,7 +16659,7 @@
       </c>
       <c r="F251" t="inlineStr" s="0">
         <is>
-          <t>Row4_GearStand_Right</t>
+          <t>STAND_ROW4_RIGHT</t>
         </is>
       </c>
       <c r="G251" t="inlineStr" s="0">
@@ -16726,7 +16726,7 @@
       </c>
       <c r="F252" t="inlineStr" s="0">
         <is>
-          <t>Row4_GearStand_Right</t>
+          <t>STAND_ROW4_RIGHT</t>
         </is>
       </c>
       <c r="G252" t="inlineStr" s="0">
@@ -16793,7 +16793,7 @@
       </c>
       <c r="F253" t="inlineStr" s="0">
         <is>
-          <t>Row4_GearStand_Right</t>
+          <t>STAND_ROW4_RIGHT</t>
         </is>
       </c>
       <c r="G253" t="inlineStr" s="0">
@@ -16860,7 +16860,7 @@
       </c>
       <c r="F254" t="inlineStr" s="0">
         <is>
-          <t>Row4_GearStand_Right</t>
+          <t>STAND_ROW4_RIGHT</t>
         </is>
       </c>
       <c r="G254" t="inlineStr" s="0">
@@ -16927,7 +16927,7 @@
       </c>
       <c r="F255" t="inlineStr" s="0">
         <is>
-          <t>Row4_GearStand_Right</t>
+          <t>STAND_ROW4_RIGHT</t>
         </is>
       </c>
       <c r="G255" t="inlineStr" s="0">
@@ -16994,7 +16994,7 @@
       </c>
       <c r="F256" t="inlineStr" s="0">
         <is>
-          <t>Row4_GearStand_Right</t>
+          <t>STAND_ROW4_RIGHT</t>
         </is>
       </c>
       <c r="G256" t="inlineStr" s="0">
@@ -17061,7 +17061,7 @@
       </c>
       <c r="F257" t="inlineStr" s="0">
         <is>
-          <t>Row4_GearStand_Right</t>
+          <t>STAND_ROW4_RIGHT</t>
         </is>
       </c>
       <c r="G257" t="inlineStr" s="0">
@@ -17128,7 +17128,7 @@
       </c>
       <c r="F258" t="inlineStr" s="0">
         <is>
-          <t>Row4_GearStand_Right</t>
+          <t>STAND_ROW4_RIGHT</t>
         </is>
       </c>
       <c r="G258" t="inlineStr" s="0">
@@ -17195,7 +17195,7 @@
       </c>
       <c r="F259" t="inlineStr" s="0">
         <is>
-          <t>Row4_GearStand_Right</t>
+          <t>STAND_ROW4_RIGHT</t>
         </is>
       </c>
       <c r="G259" t="inlineStr" s="0">
@@ -17262,7 +17262,7 @@
       </c>
       <c r="F260" t="inlineStr" s="0">
         <is>
-          <t>Row4_GearStand_Right</t>
+          <t>STAND_ROW4_RIGHT</t>
         </is>
       </c>
       <c r="G260" t="inlineStr" s="0">
@@ -17329,7 +17329,7 @@
       </c>
       <c r="F261" t="inlineStr" s="0">
         <is>
-          <t>Row4_GearStand_Right</t>
+          <t>STAND_ROW4_RIGHT</t>
         </is>
       </c>
       <c r="G261" t="inlineStr" s="0">
@@ -17396,7 +17396,7 @@
       </c>
       <c r="F262" t="inlineStr" s="0">
         <is>
-          <t>Row4_Gear_Left</t>
+          <t>GEAR_ROW4_LEFT</t>
         </is>
       </c>
       <c r="G262" t="inlineStr" s="0">
@@ -17463,7 +17463,7 @@
       </c>
       <c r="F263" t="inlineStr" s="0">
         <is>
-          <t>Row4_Gear_Left</t>
+          <t>GEAR_ROW4_LEFT</t>
         </is>
       </c>
       <c r="G263" t="inlineStr" s="0">
@@ -17530,7 +17530,7 @@
       </c>
       <c r="F264" t="inlineStr" s="0">
         <is>
-          <t>Row4_Gear_Left</t>
+          <t>GEAR_ROW4_LEFT</t>
         </is>
       </c>
       <c r="G264" t="inlineStr" s="0">
@@ -17597,7 +17597,7 @@
       </c>
       <c r="F265" t="inlineStr" s="0">
         <is>
-          <t>Row4_Gear_Left</t>
+          <t>GEAR_ROW4_LEFT</t>
         </is>
       </c>
       <c r="G265" t="inlineStr" s="0">
@@ -17664,7 +17664,7 @@
       </c>
       <c r="F266" t="inlineStr" s="0">
         <is>
-          <t>Row4_Gear_Left</t>
+          <t>GEAR_ROW4_LEFT</t>
         </is>
       </c>
       <c r="G266" t="inlineStr" s="0">
@@ -17731,7 +17731,7 @@
       </c>
       <c r="F267" t="inlineStr" s="0">
         <is>
-          <t>Row4_Gear_Left</t>
+          <t>GEAR_ROW4_LEFT</t>
         </is>
       </c>
       <c r="G267" t="inlineStr" s="0">
@@ -17798,7 +17798,7 @@
       </c>
       <c r="F268" t="inlineStr" s="0">
         <is>
-          <t>Row4_Gear_Left</t>
+          <t>GEAR_ROW4_LEFT</t>
         </is>
       </c>
       <c r="G268" t="inlineStr" s="0">
@@ -17865,7 +17865,7 @@
       </c>
       <c r="F269" t="inlineStr" s="0">
         <is>
-          <t>Row4_Gear_Left</t>
+          <t>GEAR_ROW4_LEFT</t>
         </is>
       </c>
       <c r="G269" t="inlineStr" s="0">
@@ -17932,7 +17932,7 @@
       </c>
       <c r="F270" t="inlineStr" s="0">
         <is>
-          <t>Row4_Gear_Left</t>
+          <t>GEAR_ROW4_LEFT</t>
         </is>
       </c>
       <c r="G270" t="inlineStr" s="0">
@@ -17999,7 +17999,7 @@
       </c>
       <c r="F271" t="inlineStr" s="0">
         <is>
-          <t>Row4_Gear_Left</t>
+          <t>GEAR_ROW4_LEFT</t>
         </is>
       </c>
       <c r="G271" t="inlineStr" s="0">
@@ -18066,7 +18066,7 @@
       </c>
       <c r="F272" t="inlineStr" s="0">
         <is>
-          <t>Row4_Gear_Left</t>
+          <t>GEAR_ROW4_LEFT</t>
         </is>
       </c>
       <c r="G272" t="inlineStr" s="0">
@@ -18133,7 +18133,7 @@
       </c>
       <c r="F273" t="inlineStr" s="0">
         <is>
-          <t>Row4_Gear_Left</t>
+          <t>GEAR_ROW4_LEFT</t>
         </is>
       </c>
       <c r="G273" t="inlineStr" s="0">
@@ -18200,7 +18200,7 @@
       </c>
       <c r="F274" t="inlineStr" s="0">
         <is>
-          <t>Row4_Screws</t>
+          <t>SCREW_ROW4</t>
         </is>
       </c>
       <c r="G274" t="inlineStr" s="0">
@@ -18267,7 +18267,7 @@
       </c>
       <c r="F275" t="inlineStr" s="0">
         <is>
-          <t>Row4_Screws</t>
+          <t>SCREW_ROW4</t>
         </is>
       </c>
       <c r="G275" t="inlineStr" s="0">
@@ -18334,7 +18334,7 @@
       </c>
       <c r="F276" t="inlineStr" s="0">
         <is>
-          <t>Row4_Screws</t>
+          <t>SCREW_ROW4</t>
         </is>
       </c>
       <c r="G276" t="inlineStr" s="0">
@@ -18401,7 +18401,7 @@
       </c>
       <c r="F277" t="inlineStr" s="0">
         <is>
-          <t>Row4_Screws</t>
+          <t>SCREW_ROW4</t>
         </is>
       </c>
       <c r="G277" t="inlineStr" s="0">
@@ -18468,7 +18468,7 @@
       </c>
       <c r="F278" t="inlineStr" s="0">
         <is>
-          <t>Row4_Screws</t>
+          <t>SCREW_ROW4</t>
         </is>
       </c>
       <c r="G278" t="inlineStr" s="0">
@@ -18535,7 +18535,7 @@
       </c>
       <c r="F279" t="inlineStr" s="0">
         <is>
-          <t>Row4_Screws</t>
+          <t>SCREW_ROW4</t>
         </is>
       </c>
       <c r="G279" t="inlineStr" s="0">
@@ -18602,7 +18602,7 @@
       </c>
       <c r="F280" t="inlineStr" s="0">
         <is>
-          <t>Row4_Screws</t>
+          <t>SCREW_ROW4</t>
         </is>
       </c>
       <c r="G280" t="inlineStr" s="0">
@@ -18669,7 +18669,7 @@
       </c>
       <c r="F281" t="inlineStr" s="0">
         <is>
-          <t>Row4_Screws</t>
+          <t>SCREW_ROW4</t>
         </is>
       </c>
       <c r="G281" t="inlineStr" s="0">
@@ -18736,7 +18736,7 @@
       </c>
       <c r="F282" t="inlineStr" s="0">
         <is>
-          <t>Row4_Screws</t>
+          <t>SCREW_ROW4</t>
         </is>
       </c>
       <c r="G282" t="inlineStr" s="0">
@@ -18803,7 +18803,7 @@
       </c>
       <c r="F283" t="inlineStr" s="0">
         <is>
-          <t>WoodenPin</t>
+          <t>PIN</t>
         </is>
       </c>
       <c r="G283" t="inlineStr" s="0">
@@ -18870,7 +18870,7 @@
       </c>
       <c r="F284" t="inlineStr" s="0">
         <is>
-          <t>WoodenPin</t>
+          <t>PIN</t>
         </is>
       </c>
       <c r="G284" t="inlineStr" s="0">
@@ -18937,7 +18937,7 @@
       </c>
       <c r="F285" t="inlineStr" s="0">
         <is>
-          <t>WoodenPin</t>
+          <t>PIN</t>
         </is>
       </c>
       <c r="G285" t="inlineStr" s="0">
@@ -19004,7 +19004,7 @@
       </c>
       <c r="F286" t="inlineStr" s="0">
         <is>
-          <t>WoodenPin</t>
+          <t>PIN</t>
         </is>
       </c>
       <c r="G286" t="inlineStr" s="0">
@@ -19071,7 +19071,7 @@
       </c>
       <c r="F287" t="inlineStr" s="0">
         <is>
-          <t>WoodenPin</t>
+          <t>PIN</t>
         </is>
       </c>
       <c r="G287" t="inlineStr" s="0">
@@ -19138,7 +19138,7 @@
       </c>
       <c r="F288" t="inlineStr" s="0">
         <is>
-          <t>WoodenPin</t>
+          <t>PIN</t>
         </is>
       </c>
       <c r="G288" t="inlineStr" s="0">
@@ -19205,7 +19205,7 @@
       </c>
       <c r="F289" t="inlineStr" s="0">
         <is>
-          <t>WoodenPin</t>
+          <t>PIN</t>
         </is>
       </c>
       <c r="G289" t="inlineStr" s="0">
@@ -19272,7 +19272,7 @@
       </c>
       <c r="F290" t="inlineStr" s="0">
         <is>
-          <t>WoodenPin</t>
+          <t>PIN</t>
         </is>
       </c>
       <c r="G290" t="inlineStr" s="0">
@@ -19339,7 +19339,7 @@
       </c>
       <c r="F291" t="inlineStr" s="0">
         <is>
-          <t>WoodenPin</t>
+          <t>PIN</t>
         </is>
       </c>
       <c r="G291" t="inlineStr" s="0">
@@ -19406,7 +19406,7 @@
       </c>
       <c r="F292" t="inlineStr" s="0">
         <is>
-          <t>WoodenPin</t>
+          <t>PIN</t>
         </is>
       </c>
       <c r="G292" t="inlineStr" s="0">
@@ -19445,8 +19445,142 @@
         </is>
       </c>
     </row>
+    <row r="293">
+      <c r="A293" t="inlineStr" s="0">
+        <is>
+          <t>289</t>
+        </is>
+      </c>
+      <c r="B293" t="inlineStr" s="0">
+        <is>
+          <t>2026-08-22 18:12:14</t>
+        </is>
+      </c>
+      <c r="C293" t="inlineStr" s="0">
+        <is>
+          <t>Joon</t>
+        </is>
+      </c>
+      <c r="D293" t="inlineStr" s="0">
+        <is>
+          <t>individual_part</t>
+        </is>
+      </c>
+      <c r="E293" t="inlineStr" s="0">
+        <is>
+          <t>Row1_Gear_Left.stl</t>
+        </is>
+      </c>
+      <c r="F293" t="inlineStr" s="0">
+        <is>
+          <t>GEAR_ROW1_LEFT</t>
+        </is>
+      </c>
+      <c r="G293" t="inlineStr" s="0">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="H293" t="inlineStr" s="0">
+        <is>
+          <t>The gear with circle</t>
+        </is>
+      </c>
+      <c r="I293" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J293" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="K293" t="inlineStr" s="0">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="L293" t="inlineStr" s="0">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="M293" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" t="inlineStr" s="0">
+        <is>
+          <t>290</t>
+        </is>
+      </c>
+      <c r="B294" t="inlineStr" s="0">
+        <is>
+          <t>2026-08-22 18:12:29</t>
+        </is>
+      </c>
+      <c r="C294" t="inlineStr" s="0">
+        <is>
+          <t>Joon</t>
+        </is>
+      </c>
+      <c r="D294" t="inlineStr" s="0">
+        <is>
+          <t>individual_part</t>
+        </is>
+      </c>
+      <c r="E294" t="inlineStr" s="0">
+        <is>
+          <t>Row1_Gear_Left.stl</t>
+        </is>
+      </c>
+      <c r="F294" t="inlineStr" s="0">
+        <is>
+          <t>GEAR_ROW1_LEFT</t>
+        </is>
+      </c>
+      <c r="G294" t="inlineStr" s="0">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="H294" t="inlineStr" s="0">
+        <is>
+          <t>The gear that is on the first row</t>
+        </is>
+      </c>
+      <c r="I294" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J294" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="K294" t="inlineStr" s="0">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="L294" t="inlineStr" s="0">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="M294" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:M292"/>
+  <autoFilter ref="A4:M294"/>
   <mergeCells count="3">
     <mergeCell ref="A1:M1"/>
     <mergeCell ref="A2:M2"/>

</xml_diff>